<commit_message>
mobility-theme: fix automatic docs generation for 2.0.0
</commit_message>
<xml_diff>
--- a/mobility-theme/mobility-theme.xlsx
+++ b/mobility-theme/mobility-theme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scrocca\Desktop\cefriel-github\controlled-vocabularies\base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4D28FE-B276-44CD-9620-88B5AABC2002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C2CFCE-BC47-4C00-8CB6-08DDEBD49C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -840,10 +840,10 @@
     <t>Commission Delegated Regulation (EU) 2024/490 of 29 November 2023 amending Delegated Regulation (EU) 2017/1926 supplementing Directive 2010/40/EU of the European Parliament and of the Council with regard to the provision of EU-wide multimodal travel information services</t>
   </si>
   <si>
-    <t>[CANDIDATE RELEASE] Mobility Theme</t>
-  </si>
-  <si>
     <t>Draft Controlled Vocabulary</t>
+  </si>
+  <si>
+    <t>Mobility Theme</t>
   </si>
 </sst>
 </file>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="B1" s="5" t="str">
         <f>_xlfn.CONCAT("https://w3id.org/mobilitydcat-ap/",SUBSTITUTE(LOWER(B2)," ","-"))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme</v>
       </c>
       <c r="C1" s="5"/>
     </row>
@@ -1396,7 +1396,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="B12" t="str">
         <f>_xlfn.CONCAT(B1,"/",B11)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/2.0.0</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/2.0.0</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1503,7 +1503,7 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -1538,7 +1538,7 @@
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="str">
         <f t="shared" ref="A20:A61" si="0">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B20,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>31</v>
@@ -1552,7 +1552,7 @@
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>32</v>
@@ -1562,14 +1562,14 @@
       <c r="E21" s="26"/>
       <c r="F21" s="26" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/static-road-network-data</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/static-road-network-data</v>
       </c>
       <c r="B22" s="9" t="s">
         <v>33</v>
@@ -1577,11 +1577,11 @@
       <c r="C22" s="8"/>
       <c r="E22" s="25" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A23:A32)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/geometry, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-network-geometry, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-width, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/number-of-lanes, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-number-of-lanes, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/gradients, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-gradients, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/junctions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-junctions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-classification</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/geometry, https://w3id.org/mobilitydcat-ap/mobility-theme/road-network-geometry, https://w3id.org/mobilitydcat-ap/mobility-theme/road-width, https://w3id.org/mobilitydcat-ap/mobility-theme/number-of-lanes, https://w3id.org/mobilitydcat-ap/mobility-theme/road-number-of-lanes, https://w3id.org/mobilitydcat-ap/mobility-theme/gradients, https://w3id.org/mobilitydcat-ap/mobility-theme/road-gradients, https://w3id.org/mobilitydcat-ap/mobility-theme/junctions, https://w3id.org/mobilitydcat-ap/mobility-theme/road-junctions, https://w3id.org/mobilitydcat-ap/mobility-theme/road-classification</v>
       </c>
       <c r="F22" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I22" t="s">
         <v>34</v>
@@ -1590,7 +1590,7 @@
     <row r="23" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/geometry</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/geometry</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>35</v>
@@ -1600,14 +1600,14 @@
       <c r="E23" s="17"/>
       <c r="F23" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G23" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H23" s="18" t="str">
         <f>A24</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-network-geometry</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-network-geometry</v>
       </c>
       <c r="I23" s="17" t="s">
         <v>34</v>
@@ -1616,7 +1616,7 @@
     <row r="24" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-network-geometry</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-network-geometry</v>
       </c>
       <c r="B24" s="21" t="s">
         <v>36</v>
@@ -1626,7 +1626,7 @@
       <c r="E24" s="22"/>
       <c r="F24" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H24" s="22"/>
       <c r="I24" s="22" t="s">
@@ -1636,7 +1636,7 @@
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-width</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-width</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>37</v>
@@ -1644,7 +1644,7 @@
       <c r="C25" s="7"/>
       <c r="F25" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>34</v>
@@ -1653,7 +1653,7 @@
     <row r="26" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/number-of-lanes</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/number-of-lanes</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>38</v>
@@ -1663,14 +1663,14 @@
       <c r="E26" s="17"/>
       <c r="F26" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G26" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H26" s="18" t="str">
         <f>A27</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-number-of-lanes</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-number-of-lanes</v>
       </c>
       <c r="I26" s="17" t="s">
         <v>34</v>
@@ -1679,7 +1679,7 @@
     <row r="27" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-number-of-lanes</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-number-of-lanes</v>
       </c>
       <c r="B27" s="21" t="s">
         <v>39</v>
@@ -1689,7 +1689,7 @@
       <c r="E27" s="22"/>
       <c r="F27" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H27" s="22"/>
       <c r="I27" s="22" t="s">
@@ -1699,7 +1699,7 @@
     <row r="28" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/gradients</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/gradients</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>40</v>
@@ -1709,14 +1709,14 @@
       <c r="E28" s="17"/>
       <c r="F28" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G28" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H28" s="18" t="str">
         <f>A29</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-gradients</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-gradients</v>
       </c>
       <c r="I28" s="17" t="s">
         <v>34</v>
@@ -1725,7 +1725,7 @@
     <row r="29" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-gradients</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-gradients</v>
       </c>
       <c r="B29" s="21" t="s">
         <v>41</v>
@@ -1735,7 +1735,7 @@
       <c r="E29" s="22"/>
       <c r="F29" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H29" s="22"/>
       <c r="I29" s="22" t="s">
@@ -1745,7 +1745,7 @@
     <row r="30" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/junctions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/junctions</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>42</v>
@@ -1755,14 +1755,14 @@
       <c r="E30" s="17"/>
       <c r="F30" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G30" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H30" s="18" t="str">
         <f>A31</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-junctions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-junctions</v>
       </c>
       <c r="I30" s="17" t="s">
         <v>34</v>
@@ -1771,7 +1771,7 @@
     <row r="31" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-junctions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-junctions</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>43</v>
@@ -1781,7 +1781,7 @@
       <c r="E31" s="22"/>
       <c r="F31" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H31" s="22"/>
       <c r="I31" s="22" t="s">
@@ -1791,7 +1791,7 @@
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-classification</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-classification</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>44</v>
@@ -1799,16 +1799,16 @@
       <c r="C32" s="7"/>
       <c r="F32" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/cycle-network-data</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/cycle-network-data</v>
       </c>
       <c r="B33" s="9" t="s">
         <v>45</v>
@@ -1816,11 +1816,11 @@
       <c r="C33" s="8"/>
       <c r="E33" s="25" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A34:A39)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/network-geometry-and-lane-character, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/cycle-network-geometry, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/network-detailed-attributes, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/cycle-network-detailed-attributes, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/network-closures-diversions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/cycle-network-closures-diversions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/network-geometry-and-lane-character, https://w3id.org/mobilitydcat-ap/mobility-theme/cycle-network-geometry, https://w3id.org/mobilitydcat-ap/mobility-theme/network-detailed-attributes, https://w3id.org/mobilitydcat-ap/mobility-theme/cycle-network-detailed-attributes, https://w3id.org/mobilitydcat-ap/mobility-theme/network-closures-diversions, https://w3id.org/mobilitydcat-ap/mobility-theme/cycle-network-closures-diversions</v>
       </c>
       <c r="F33" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>46</v>
@@ -1829,7 +1829,7 @@
     <row r="34" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/network-geometry-and-lane-character</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/network-geometry-and-lane-character</v>
       </c>
       <c r="B34" s="16" t="s">
         <v>47</v>
@@ -1839,7 +1839,7 @@
       <c r="E34" s="17"/>
       <c r="F34" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G34" s="18" t="b">
         <v>1</v>
@@ -1851,10 +1851,10 @@
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B35,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/cycle-network-geometry</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/cycle-network-geometry</v>
       </c>
       <c r="B35" s="24" t="s">
         <v>49</v>
@@ -1866,7 +1866,7 @@
       <c r="E35" s="22"/>
       <c r="F35" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H35" s="22"/>
       <c r="I35" s="22" t="s">
@@ -1876,7 +1876,7 @@
     <row r="36" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="str">
         <f t="shared" ref="A36" si="1">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B36,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/network-detailed-attributes</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/network-detailed-attributes</v>
       </c>
       <c r="B36" s="16" t="s">
         <v>51</v>
@@ -1886,7 +1886,7 @@
       <c r="E36" s="17"/>
       <c r="F36" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G36" s="18" t="b">
         <v>1</v>
@@ -1901,7 +1901,7 @@
     <row r="37" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/cycle-network-detailed-attributes</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/cycle-network-detailed-attributes</v>
       </c>
       <c r="B37" s="24" t="s">
         <v>53</v>
@@ -1911,7 +1911,7 @@
       <c r="E37" s="22"/>
       <c r="F37" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H37" s="22"/>
       <c r="I37" s="22" t="s">
@@ -1921,7 +1921,7 @@
     <row r="38" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B38,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/network-closures-diversions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/network-closures-diversions</v>
       </c>
       <c r="B38" s="16" t="s">
         <v>54</v>
@@ -1931,7 +1931,7 @@
       <c r="E38" s="17"/>
       <c r="F38" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G38" s="18" t="b">
         <v>1</v>
@@ -1944,7 +1944,7 @@
     <row r="39" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="20" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B39,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/cycle-network-closures-diversions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/cycle-network-closures-diversions</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>56</v>
@@ -1954,15 +1954,15 @@
       <c r="E39" s="22"/>
       <c r="F39" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H39" s="22"/>
       <c r="I39" s="22"/>
     </row>
-    <row r="40" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/pedestrian-network-data</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/pedestrian-network-data</v>
       </c>
       <c r="B40" s="9" t="s">
         <v>57</v>
@@ -1970,11 +1970,11 @@
       <c r="C40" s="8"/>
       <c r="E40" s="1" t="str">
         <f>CONCATENATE(A41,", ",A42)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/pedestrian-network-geometry, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/pedestrian-accessibility-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/pedestrian-network-geometry, https://w3id.org/mobilitydcat-ap/mobility-theme/pedestrian-accessibility-facilities</v>
       </c>
       <c r="F40" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>46</v>
@@ -1983,7 +1983,7 @@
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/pedestrian-network-geometry</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/pedestrian-network-geometry</v>
       </c>
       <c r="B41" s="13" t="s">
         <v>58</v>
@@ -1991,7 +1991,7 @@
       <c r="C41" s="8"/>
       <c r="F41" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>46</v>
@@ -2000,7 +2000,7 @@
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/pedestrian-accessibility-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/pedestrian-accessibility-facilities</v>
       </c>
       <c r="B42" s="13" t="s">
         <v>59</v>
@@ -2008,7 +2008,7 @@
       <c r="C42" s="8"/>
       <c r="F42" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>46</v>
@@ -2017,7 +2017,7 @@
     <row r="43" spans="1:9" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/static-traffic-signs-and-regulations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/static-traffic-signs-and-regulations</v>
       </c>
       <c r="B43" s="9" t="s">
         <v>60</v>
@@ -2025,11 +2025,11 @@
       <c r="C43" s="8"/>
       <c r="E43" s="25" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A44:A54)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/tunnel-access-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bridge-access-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/speed-limits, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other-static-traffic-signs, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/permanent-access-restrictions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other-traffic-regulations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/traffic-circulation-plans, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/static-overtaking-bans-on-heavy-goods-vehicles, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/weight-length-width-height-restrictions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/one-way-streets, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/regulated-traffic-zones</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/tunnel-access-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/bridge-access-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/speed-limits, https://w3id.org/mobilitydcat-ap/mobility-theme/other-static-traffic-signs, https://w3id.org/mobilitydcat-ap/mobility-theme/permanent-access-restrictions, https://w3id.org/mobilitydcat-ap/mobility-theme/other-traffic-regulations, https://w3id.org/mobilitydcat-ap/mobility-theme/traffic-circulation-plans, https://w3id.org/mobilitydcat-ap/mobility-theme/static-overtaking-bans-on-heavy-goods-vehicles, https://w3id.org/mobilitydcat-ap/mobility-theme/weight-length-width-height-restrictions, https://w3id.org/mobilitydcat-ap/mobility-theme/one-way-streets, https://w3id.org/mobilitydcat-ap/mobility-theme/regulated-traffic-zones</v>
       </c>
       <c r="F43" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>34</v>
@@ -2038,7 +2038,7 @@
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/tunnel-access-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/tunnel-access-conditions</v>
       </c>
       <c r="B44" s="8" t="s">
         <v>61</v>
@@ -2046,7 +2046,7 @@
       <c r="C44" s="8"/>
       <c r="F44" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>34</v>
@@ -2055,7 +2055,7 @@
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bridge-access-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/bridge-access-conditions</v>
       </c>
       <c r="B45" s="8" t="s">
         <v>62</v>
@@ -2063,7 +2063,7 @@
       <c r="C45" s="8"/>
       <c r="F45" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>34</v>
@@ -2072,7 +2072,7 @@
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/speed-limits</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/speed-limits</v>
       </c>
       <c r="B46" s="8" t="s">
         <v>63</v>
@@ -2080,7 +2080,7 @@
       <c r="C46" s="8"/>
       <c r="F46" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I46" s="1" t="s">
         <v>34</v>
@@ -2089,7 +2089,7 @@
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other-static-traffic-signs</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/other-static-traffic-signs</v>
       </c>
       <c r="B47" s="8" t="s">
         <v>64</v>
@@ -2097,7 +2097,7 @@
       <c r="C47" s="8"/>
       <c r="F47" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I47" s="25" t="s">
         <v>34</v>
@@ -2106,7 +2106,7 @@
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/permanent-access-restrictions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/permanent-access-restrictions</v>
       </c>
       <c r="B48" s="8" t="s">
         <v>65</v>
@@ -2114,7 +2114,7 @@
       <c r="C48" s="8"/>
       <c r="F48" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>34</v>
@@ -2123,7 +2123,7 @@
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other-traffic-regulations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/other-traffic-regulations</v>
       </c>
       <c r="B49" s="8" t="s">
         <v>66</v>
@@ -2131,7 +2131,7 @@
       <c r="C49" s="8"/>
       <c r="F49" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I49" s="1" t="s">
         <v>34</v>
@@ -2140,7 +2140,7 @@
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/traffic-circulation-plans</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/traffic-circulation-plans</v>
       </c>
       <c r="B50" s="8" t="s">
         <v>67</v>
@@ -2148,7 +2148,7 @@
       <c r="C50" s="8"/>
       <c r="F50" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>34</v>
@@ -2157,7 +2157,7 @@
     <row r="51" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/static-overtaking-bans-on-heavy-goods-vehicles</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/static-overtaking-bans-on-heavy-goods-vehicles</v>
       </c>
       <c r="B51" s="24" t="s">
         <v>68</v>
@@ -2167,7 +2167,7 @@
       <c r="E51" s="22"/>
       <c r="F51" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H51" s="22"/>
       <c r="I51" s="22" t="s">
@@ -2177,7 +2177,7 @@
     <row r="52" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/weight-length-width-height-restrictions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/weight-length-width-height-restrictions</v>
       </c>
       <c r="B52" s="24" t="s">
         <v>69</v>
@@ -2187,7 +2187,7 @@
       <c r="E52" s="22"/>
       <c r="F52" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H52" s="22"/>
       <c r="I52" s="22" t="s">
@@ -2197,7 +2197,7 @@
     <row r="53" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/one-way-streets</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/one-way-streets</v>
       </c>
       <c r="B53" s="24" t="s">
         <v>70</v>
@@ -2207,7 +2207,7 @@
       <c r="E53" s="22"/>
       <c r="F53" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H53" s="22"/>
       <c r="I53" s="22" t="s">
@@ -2217,7 +2217,7 @@
     <row r="54" spans="1:9" s="23" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A54" s="20" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/regulated-traffic-zones</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/regulated-traffic-zones</v>
       </c>
       <c r="B54" s="24" t="s">
         <v>71</v>
@@ -2229,17 +2229,17 @@
       <c r="E54" s="22"/>
       <c r="F54" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H54" s="22"/>
       <c r="I54" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/toll-information</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/toll-information</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>73</v>
@@ -2247,11 +2247,11 @@
       <c r="C55" s="8"/>
       <c r="E55" s="25" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A56:A61)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/location-of-tolling-stations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/identification-of-tolled-roads, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/applicable-road-user-charges-and-payment-methods, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/fixed-road-user-charges-and-payment-methods, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/variable-road-user-charges-and-payment-methods, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/payment-methods-for-tolls</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/location-of-tolling-stations, https://w3id.org/mobilitydcat-ap/mobility-theme/identification-of-tolled-roads, https://w3id.org/mobilitydcat-ap/mobility-theme/applicable-road-user-charges-and-payment-methods, https://w3id.org/mobilitydcat-ap/mobility-theme/fixed-road-user-charges-and-payment-methods, https://w3id.org/mobilitydcat-ap/mobility-theme/variable-road-user-charges-and-payment-methods, https://w3id.org/mobilitydcat-ap/mobility-theme/payment-methods-for-tolls</v>
       </c>
       <c r="F55" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>34</v>
@@ -2260,7 +2260,7 @@
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/location-of-tolling-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/location-of-tolling-stations</v>
       </c>
       <c r="B56" s="8" t="s">
         <v>74</v>
@@ -2268,7 +2268,7 @@
       <c r="C56" s="8"/>
       <c r="F56" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I56" s="1" t="s">
         <v>34</v>
@@ -2277,7 +2277,7 @@
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/identification-of-tolled-roads</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/identification-of-tolled-roads</v>
       </c>
       <c r="B57" s="8" t="s">
         <v>75</v>
@@ -2285,7 +2285,7 @@
       <c r="C57" s="8"/>
       <c r="F57" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>34</v>
@@ -2294,7 +2294,7 @@
     <row r="58" spans="1:9" s="18" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/applicable-road-user-charges-and-payment-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/applicable-road-user-charges-and-payment-methods</v>
       </c>
       <c r="B58" s="16" t="s">
         <v>76</v>
@@ -2304,14 +2304,14 @@
       <c r="E58" s="17"/>
       <c r="F58" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G58" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H58" s="17" t="str">
         <f>A59</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/fixed-road-user-charges-and-payment-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/fixed-road-user-charges-and-payment-methods</v>
       </c>
       <c r="I58" s="18" t="s">
         <v>34</v>
@@ -2320,7 +2320,7 @@
     <row r="59" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="20" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B59,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/fixed-road-user-charges-and-payment-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/fixed-road-user-charges-and-payment-methods</v>
       </c>
       <c r="B59" s="24" t="s">
         <v>77</v>
@@ -2330,7 +2330,7 @@
       <c r="E59" s="22"/>
       <c r="F59" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H59" s="22"/>
       <c r="I59" s="23" t="s">
@@ -2340,7 +2340,7 @@
     <row r="60" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="20" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B60,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/variable-road-user-charges-and-payment-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/variable-road-user-charges-and-payment-methods</v>
       </c>
       <c r="B60" s="24" t="s">
         <v>78</v>
@@ -2350,7 +2350,7 @@
       <c r="E60" s="22"/>
       <c r="F60" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H60" s="22"/>
       <c r="I60" s="23" t="s">
@@ -2360,7 +2360,7 @@
     <row r="61" spans="1:9" s="18" customFormat="1" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/payment-methods-for-tolls</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/payment-methods-for-tolls</v>
       </c>
       <c r="B61" s="16" t="s">
         <v>79</v>
@@ -2370,14 +2370,14 @@
       <c r="E61" s="17"/>
       <c r="F61" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G61" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H61" s="17" t="str">
         <f>_xlfn.CONCAT(A59,",",A60)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/fixed-road-user-charges-and-payment-methods,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/variable-road-user-charges-and-payment-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/fixed-road-user-charges-and-payment-methods,https://w3id.org/mobilitydcat-ap/mobility-theme/variable-road-user-charges-and-payment-methods</v>
       </c>
       <c r="I61" s="17" t="s">
         <v>34</v>
@@ -2386,7 +2386,7 @@
     <row r="62" spans="1:9" ht="144" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B62,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-service-and-rest-area-information</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-service-and-rest-area-information</v>
       </c>
       <c r="B62" s="9" t="s">
         <v>80</v>
@@ -2394,20 +2394,20 @@
       <c r="C62" s="8"/>
       <c r="E62" s="25" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A63:A79)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-parking-locations-and-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-parking-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-locations-description-and-facilities, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-zones, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-real-time-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-conditions-and-tariffs, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-payment-points-and-methods, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-locations-and-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-locations-description-and-facilities, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-real-time-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/truck-parking-locations-and-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/truck-parking-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/park-and-ride-stops, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/park-and-drive-stops, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/kiss-and-ride-stops, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-parking-locations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/car-parking-locations-and-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/car-parking-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/parking-locations-description-and-facilities, https://w3id.org/mobilitydcat-ap/mobility-theme/parking-zones, https://w3id.org/mobilitydcat-ap/mobility-theme/parking-real-time-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/parking-conditions-and-tariffs, https://w3id.org/mobilitydcat-ap/mobility-theme/parking-payment-points-and-methods, https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-locations-and-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-locations-description-and-facilities, https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-real-time-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/truck-parking-locations-and-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/truck-parking-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/park-and-ride-stops, https://w3id.org/mobilitydcat-ap/mobility-theme/park-and-drive-stops, https://w3id.org/mobilitydcat-ap/mobility-theme/kiss-and-ride-stops, https://w3id.org/mobilitydcat-ap/mobility-theme/bike-parking-locations</v>
       </c>
       <c r="F62" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="63" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A63" s="15" t="str">
         <f t="shared" ref="A63:A150" si="2">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B63,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-parking-locations-and-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/car-parking-locations-and-conditions</v>
       </c>
       <c r="B63" s="16" t="s">
         <v>82</v>
@@ -2417,23 +2417,23 @@
       <c r="E63" s="17"/>
       <c r="F63" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G63" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H63" s="17" t="str">
         <f>A65</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-locations-description-and-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-locations-description-and-facilities</v>
       </c>
       <c r="I63" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="64" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-parking-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/car-parking-availability</v>
       </c>
       <c r="B64" s="16" t="s">
         <v>83</v>
@@ -2443,14 +2443,14 @@
       <c r="E64" s="17"/>
       <c r="F64" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G64" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H64" s="17" t="str">
         <f>A67</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-real-time-availability</v>
       </c>
       <c r="I64" s="17" t="s">
         <v>46</v>
@@ -2459,7 +2459,7 @@
     <row r="65" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-locations-description-and-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-locations-description-and-facilities</v>
       </c>
       <c r="B65" s="24" t="s">
         <v>84</v>
@@ -2469,7 +2469,7 @@
       <c r="E65" s="22"/>
       <c r="F65" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H65" s="22"/>
       <c r="I65" s="22"/>
@@ -2477,7 +2477,7 @@
     <row r="66" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-zones</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-zones</v>
       </c>
       <c r="B66" s="24" t="s">
         <v>85</v>
@@ -2487,7 +2487,7 @@
       <c r="E66" s="22"/>
       <c r="F66" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H66" s="22"/>
       <c r="I66" s="22"/>
@@ -2495,7 +2495,7 @@
     <row r="67" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-real-time-availability</v>
       </c>
       <c r="B67" s="24" t="s">
         <v>86</v>
@@ -2505,7 +2505,7 @@
       <c r="E67" s="22"/>
       <c r="F67" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H67" s="22"/>
       <c r="I67" s="22"/>
@@ -2513,7 +2513,7 @@
     <row r="68" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-conditions-and-tariffs</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-conditions-and-tariffs</v>
       </c>
       <c r="B68" s="24" t="s">
         <v>87</v>
@@ -2523,7 +2523,7 @@
       <c r="E68" s="22"/>
       <c r="F68" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H68" s="22"/>
       <c r="I68" s="22"/>
@@ -2531,7 +2531,7 @@
     <row r="69" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-payment-points-and-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-payment-points-and-methods</v>
       </c>
       <c r="B69" s="24" t="s">
         <v>88</v>
@@ -2543,7 +2543,7 @@
       <c r="E69" s="22"/>
       <c r="F69" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H69" s="22"/>
       <c r="I69" s="22"/>
@@ -2551,7 +2551,7 @@
     <row r="70" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-locations-and-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-locations-and-conditions</v>
       </c>
       <c r="B70" s="16" t="s">
         <v>90</v>
@@ -2561,14 +2561,14 @@
       <c r="E70" s="17"/>
       <c r="F70" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G70" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H70" s="17" t="str">
         <f>A71</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-locations-description-and-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-locations-description-and-facilities</v>
       </c>
       <c r="I70" s="17" t="s">
         <v>34</v>
@@ -2577,7 +2577,7 @@
     <row r="71" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-locations-description-and-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-locations-description-and-facilities</v>
       </c>
       <c r="B71" s="24" t="s">
         <v>91</v>
@@ -2587,15 +2587,15 @@
       <c r="E71" s="22"/>
       <c r="F71" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H71" s="22"/>
       <c r="I71" s="22"/>
     </row>
-    <row r="72" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-availability</v>
       </c>
       <c r="B72" s="16" t="s">
         <v>92</v>
@@ -2605,21 +2605,21 @@
       <c r="E72" s="17"/>
       <c r="F72" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G72" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H72" s="17" t="str">
         <f>A73</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-real-time-availability</v>
       </c>
       <c r="I72" s="17"/>
     </row>
     <row r="73" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-and-rest-area-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-and-rest-area-real-time-availability</v>
       </c>
       <c r="B73" s="24" t="s">
         <v>93</v>
@@ -2629,15 +2629,15 @@
       <c r="E73" s="22"/>
       <c r="F73" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H73" s="22"/>
       <c r="I73" s="22"/>
     </row>
-    <row r="74" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/truck-parking-locations-and-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/truck-parking-locations-and-conditions</v>
       </c>
       <c r="B74" s="16" t="s">
         <v>94</v>
@@ -2647,23 +2647,23 @@
       <c r="E74" s="17"/>
       <c r="F74" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G74" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H74" s="17" t="str">
         <f>A65</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-locations-description-and-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-locations-description-and-facilities</v>
       </c>
       <c r="I74" s="17" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="75" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/truck-parking-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/truck-parking-availability</v>
       </c>
       <c r="B75" s="16" t="s">
         <v>96</v>
@@ -2673,23 +2673,23 @@
       <c r="E75" s="17"/>
       <c r="F75" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G75" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H75" s="17" t="str">
         <f>A67</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-real-time-availability</v>
       </c>
       <c r="I75" s="17" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/park-and-ride-stops</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/park-and-ride-stops</v>
       </c>
       <c r="B76" s="8" t="s">
         <v>97</v>
@@ -2700,16 +2700,16 @@
       </c>
       <c r="F76" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I76" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="77" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/park-and-drive-stops</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/park-and-drive-stops</v>
       </c>
       <c r="B77" s="24" t="s">
         <v>99</v>
@@ -2721,7 +2721,7 @@
       <c r="E77" s="22"/>
       <c r="F77" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H77" s="22"/>
       <c r="I77" s="22" t="s">
@@ -2731,7 +2731,7 @@
     <row r="78" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/kiss-and-ride-stops</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/kiss-and-ride-stops</v>
       </c>
       <c r="B78" s="24" t="s">
         <v>101</v>
@@ -2741,15 +2741,15 @@
       <c r="E78" s="22"/>
       <c r="F78" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H78" s="22"/>
       <c r="I78" s="22"/>
     </row>
-    <row r="79" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-parking-locations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/bike-parking-locations</v>
       </c>
       <c r="B79" s="16" t="s">
         <v>102</v>
@@ -2759,14 +2759,14 @@
       <c r="E79" s="17"/>
       <c r="F79" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G79" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H79" s="17" t="str">
         <f>A65</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parking-locations-description-and-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parking-locations-description-and-facilities</v>
       </c>
       <c r="I79" s="17" t="s">
         <v>46</v>
@@ -2775,7 +2775,7 @@
     <row r="80" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/filling-and-charging-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/filling-and-charging-stations</v>
       </c>
       <c r="B80" s="9" t="s">
         <v>103</v>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="F80" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I80" s="25" t="s">
         <v>104</v>
@@ -2796,7 +2796,7 @@
     <row r="81" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/location-and-conditions-of-charging-points</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/location-and-conditions-of-charging-points</v>
       </c>
       <c r="B81" s="16" t="s">
         <v>105</v>
@@ -2806,7 +2806,7 @@
       <c r="E81" s="17"/>
       <c r="F81" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G81" s="18" t="b">
         <v>1</v>
@@ -2822,7 +2822,7 @@
     <row r="82" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/location-and-conditions-of-filling-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/location-and-conditions-of-filling-stations</v>
       </c>
       <c r="B82" s="16" t="s">
         <v>106</v>
@@ -2832,7 +2832,7 @@
       <c r="E82" s="17"/>
       <c r="F82" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G82" s="18" t="b">
         <v>1</v>
@@ -2848,7 +2848,7 @@
     <row r="83" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/availability-of-charging-points-for-electric-vehicles</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/availability-of-charging-points-for-electric-vehicles</v>
       </c>
       <c r="B83" s="16" t="s">
         <v>107</v>
@@ -2858,7 +2858,7 @@
       <c r="E83" s="17"/>
       <c r="F83" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G83" s="18" t="b">
         <v>1</v>
@@ -2874,7 +2874,7 @@
     <row r="84" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/availability-of-filling-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/availability-of-filling-stations</v>
       </c>
       <c r="B84" s="16" t="s">
         <v>108</v>
@@ -2884,7 +2884,7 @@
       <c r="E84" s="17"/>
       <c r="F84" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G84" s="18" t="b">
         <v>1</v>
@@ -2909,7 +2909,7 @@
       <c r="E85" s="22"/>
       <c r="F85" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H85" s="22"/>
       <c r="I85" s="22" t="s">
@@ -2928,7 +2928,7 @@
       <c r="E86" s="22"/>
       <c r="F86" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H86" s="22"/>
       <c r="I86" s="22" t="s">
@@ -2947,17 +2947,17 @@
       <c r="E87" s="22"/>
       <c r="F87" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H87" s="22"/>
       <c r="I87" s="22" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A88" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/freight-and-logistics</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/freight-and-logistics</v>
       </c>
       <c r="B88" s="9" t="s">
         <v>115</v>
@@ -2965,11 +2965,11 @@
       <c r="C88" s="8"/>
       <c r="E88" s="1" t="str">
         <f>CONCATENATE(A89,", ",A90,", ",A91)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/freight-delivery-regulations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/location-of-delivery-areas, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/availability-of-delivery-areas</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/freight-delivery-regulations, https://w3id.org/mobilitydcat-ap/mobility-theme/location-of-delivery-areas, https://w3id.org/mobilitydcat-ap/mobility-theme/availability-of-delivery-areas</v>
       </c>
       <c r="F88" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I88" s="1" t="s">
         <v>34</v>
@@ -2978,7 +2978,7 @@
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/freight-delivery-regulations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/freight-delivery-regulations</v>
       </c>
       <c r="B89" s="8" t="s">
         <v>116</v>
@@ -2986,7 +2986,7 @@
       <c r="C89" s="8"/>
       <c r="F89" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I89" s="1" t="s">
         <v>34</v>
@@ -2995,7 +2995,7 @@
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/location-of-delivery-areas</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/location-of-delivery-areas</v>
       </c>
       <c r="B90" s="8" t="s">
         <v>117</v>
@@ -3003,7 +3003,7 @@
       <c r="C90" s="8"/>
       <c r="F90" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I90" s="1" t="s">
         <v>34</v>
@@ -3012,7 +3012,7 @@
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/availability-of-delivery-areas</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/availability-of-delivery-areas</v>
       </c>
       <c r="B91" s="8" t="s">
         <v>118</v>
@@ -3020,16 +3020,16 @@
       <c r="C91" s="8"/>
       <c r="F91" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I91" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" ht="165" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/dynamic-traffic-signs-and-regulations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/dynamic-traffic-signs-and-regulations</v>
       </c>
       <c r="B92" s="9" t="s">
         <v>119</v>
@@ -3037,11 +3037,11 @@
       <c r="C92" s="8"/>
       <c r="E92" s="1" t="str">
         <f>CONCATENATE(A93,", ",A94,", ",A95,", ",A96,", ",A97,", ",A98,", ",A99,", ",A100,", ",A101)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-closures-and-access-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/lane-closures-and-access-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bridge-closures-and-access-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/tunnel-closures-and-access-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other-access-restrictions-and-traffic-regulations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/dynamic-overtaking-bans-on-heavy-goods-vehicles, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/dynamic-speed-limits, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/direction-of-travel-on-reversible-lanes, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other-temporary-traffic-management-measures-or-plans</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-closures-and-access-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/lane-closures-and-access-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/bridge-closures-and-access-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/tunnel-closures-and-access-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/other-access-restrictions-and-traffic-regulations, https://w3id.org/mobilitydcat-ap/mobility-theme/dynamic-overtaking-bans-on-heavy-goods-vehicles, https://w3id.org/mobilitydcat-ap/mobility-theme/dynamic-speed-limits, https://w3id.org/mobilitydcat-ap/mobility-theme/direction-of-travel-on-reversible-lanes, https://w3id.org/mobilitydcat-ap/mobility-theme/other-temporary-traffic-management-measures-or-plans</v>
       </c>
       <c r="F92" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I92" s="1" t="s">
         <v>34</v>
@@ -3050,7 +3050,7 @@
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-closures-and-access-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-closures-and-access-conditions</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>120</v>
@@ -3058,7 +3058,7 @@
       <c r="C93" s="8"/>
       <c r="F93" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I93" s="1" t="s">
         <v>34</v>
@@ -3067,7 +3067,7 @@
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/lane-closures-and-access-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/lane-closures-and-access-conditions</v>
       </c>
       <c r="B94" s="8" t="s">
         <v>121</v>
@@ -3075,7 +3075,7 @@
       <c r="C94" s="8"/>
       <c r="F94" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I94" s="1" t="s">
         <v>34</v>
@@ -3084,7 +3084,7 @@
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bridge-closures-and-access-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/bridge-closures-and-access-conditions</v>
       </c>
       <c r="B95" s="8" t="s">
         <v>122</v>
@@ -3092,7 +3092,7 @@
       <c r="C95" s="8"/>
       <c r="F95" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I95" s="1" t="s">
         <v>34</v>
@@ -3101,7 +3101,7 @@
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/tunnel-closures-and-access-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/tunnel-closures-and-access-conditions</v>
       </c>
       <c r="B96" s="8" t="s">
         <v>123</v>
@@ -3109,7 +3109,7 @@
       <c r="C96" s="8"/>
       <c r="F96" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I96" s="1" t="s">
         <v>34</v>
@@ -3118,7 +3118,7 @@
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other-access-restrictions-and-traffic-regulations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/other-access-restrictions-and-traffic-regulations</v>
       </c>
       <c r="B97" s="8" t="s">
         <v>124</v>
@@ -3126,7 +3126,7 @@
       <c r="C97" s="8"/>
       <c r="F97" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I97" s="1" t="s">
         <v>34</v>
@@ -3135,7 +3135,7 @@
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/dynamic-overtaking-bans-on-heavy-goods-vehicles</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/dynamic-overtaking-bans-on-heavy-goods-vehicles</v>
       </c>
       <c r="B98" s="8" t="s">
         <v>125</v>
@@ -3143,7 +3143,7 @@
       <c r="C98" s="8"/>
       <c r="F98" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I98" s="1" t="s">
         <v>34</v>
@@ -3152,7 +3152,7 @@
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/dynamic-speed-limits</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/dynamic-speed-limits</v>
       </c>
       <c r="B99" s="8" t="s">
         <v>126</v>
@@ -3160,7 +3160,7 @@
       <c r="C99" s="8"/>
       <c r="F99" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I99" s="1" t="s">
         <v>34</v>
@@ -3169,7 +3169,7 @@
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/direction-of-travel-on-reversible-lanes</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/direction-of-travel-on-reversible-lanes</v>
       </c>
       <c r="B100" s="8" t="s">
         <v>127</v>
@@ -3177,7 +3177,7 @@
       <c r="C100" s="8"/>
       <c r="F100" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I100" s="1" t="s">
         <v>34</v>
@@ -3186,7 +3186,7 @@
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other-temporary-traffic-management-measures-or-plans</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/other-temporary-traffic-management-measures-or-plans</v>
       </c>
       <c r="B101" s="8" t="s">
         <v>128</v>
@@ -3194,7 +3194,7 @@
       <c r="C101" s="8"/>
       <c r="F101" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I101" s="1" t="s">
         <v>34</v>
@@ -3203,7 +3203,7 @@
     <row r="102" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A102" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-work-information</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-work-information</v>
       </c>
       <c r="B102" s="9" t="s">
         <v>129</v>
@@ -3211,11 +3211,11 @@
       <c r="C102" s="8"/>
       <c r="E102" s="1" t="str">
         <f>CONCATENATE(A103,", ",A104)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/long-term-road-works, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/short-term-road-works</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/long-term-road-works, https://w3id.org/mobilitydcat-ap/mobility-theme/short-term-road-works</v>
       </c>
       <c r="F102" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I102" s="1" t="s">
         <v>130</v>
@@ -3224,7 +3224,7 @@
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/long-term-road-works</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/long-term-road-works</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>131</v>
@@ -3232,7 +3232,7 @@
       <c r="C103" s="8"/>
       <c r="F103" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I103" s="1" t="s">
         <v>34</v>
@@ -3241,7 +3241,7 @@
     <row r="104" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/short-term-road-works</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/short-term-road-works</v>
       </c>
       <c r="B104" s="8" t="s">
         <v>132</v>
@@ -3249,7 +3249,7 @@
       <c r="C104" s="8"/>
       <c r="F104" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I104" s="1" t="s">
         <v>130</v>
@@ -3258,7 +3258,7 @@
     <row r="105" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A105" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-events-and-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-events-and-conditions</v>
       </c>
       <c r="B105" s="9" t="s">
         <v>133</v>
@@ -3266,11 +3266,11 @@
       <c r="C105" s="8"/>
       <c r="E105" s="1" t="str">
         <f>CONCATENATE(A106,", ",A107,", ",A108)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/accidents-and-incidents, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/poor-road-conditions, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-weather-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/accidents-and-incidents, https://w3id.org/mobilitydcat-ap/mobility-theme/poor-road-conditions, https://w3id.org/mobilitydcat-ap/mobility-theme/road-weather-conditions</v>
       </c>
       <c r="F105" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I105" s="1" t="s">
         <v>130</v>
@@ -3279,7 +3279,7 @@
     <row r="106" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/accidents-and-incidents</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/accidents-and-incidents</v>
       </c>
       <c r="B106" s="8" t="s">
         <v>134</v>
@@ -3287,7 +3287,7 @@
       <c r="C106" s="8"/>
       <c r="F106" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I106" s="1" t="s">
         <v>130</v>
@@ -3296,7 +3296,7 @@
     <row r="107" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A107" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/poor-road-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/poor-road-conditions</v>
       </c>
       <c r="B107" s="8" t="s">
         <v>135</v>
@@ -3304,7 +3304,7 @@
       <c r="C107" s="8"/>
       <c r="F107" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I107" s="1" t="s">
         <v>130</v>
@@ -3313,7 +3313,7 @@
     <row r="108" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A108" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/road-weather-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/road-weather-conditions</v>
       </c>
       <c r="B108" s="8" t="s">
         <v>136</v>
@@ -3321,16 +3321,16 @@
       <c r="C108" s="8"/>
       <c r="F108" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I108" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" ht="195" x14ac:dyDescent="0.25">
       <c r="A109" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/real-time-traffic-data</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/real-time-traffic-data</v>
       </c>
       <c r="B109" s="9" t="s">
         <v>137</v>
@@ -3338,11 +3338,11 @@
       <c r="C109" s="8"/>
       <c r="E109" s="25" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A110:A121)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/traffic-volume, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/speed, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/traffic-speed, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/location-and-length-of-traffic-queues, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/current-travel-times, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/current-road-travel-times, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/predicted-travel-times, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/predicted-road-travel-times, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/expected-delays, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/expected-road-traffic-delays, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/waiting-time-at-border-crossings-to-non-eu-member-states, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/traffic-data-at-border-crossings-to-third-countries</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/traffic-volume, https://w3id.org/mobilitydcat-ap/mobility-theme/speed, https://w3id.org/mobilitydcat-ap/mobility-theme/traffic-speed, https://w3id.org/mobilitydcat-ap/mobility-theme/location-and-length-of-traffic-queues, https://w3id.org/mobilitydcat-ap/mobility-theme/current-travel-times, https://w3id.org/mobilitydcat-ap/mobility-theme/current-road-travel-times, https://w3id.org/mobilitydcat-ap/mobility-theme/predicted-travel-times, https://w3id.org/mobilitydcat-ap/mobility-theme/predicted-road-travel-times, https://w3id.org/mobilitydcat-ap/mobility-theme/expected-delays, https://w3id.org/mobilitydcat-ap/mobility-theme/expected-road-traffic-delays, https://w3id.org/mobilitydcat-ap/mobility-theme/waiting-time-at-border-crossings-to-non-eu-member-states, https://w3id.org/mobilitydcat-ap/mobility-theme/traffic-data-at-border-crossings-to-third-countries</v>
       </c>
       <c r="F109" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I109" s="1" t="s">
         <v>34</v>
@@ -3351,7 +3351,7 @@
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/traffic-volume</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/traffic-volume</v>
       </c>
       <c r="B110" s="8" t="s">
         <v>138</v>
@@ -3359,7 +3359,7 @@
       <c r="C110" s="8"/>
       <c r="F110" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I110" s="1" t="s">
         <v>34</v>
@@ -3368,7 +3368,7 @@
     <row r="111" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/speed</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/speed</v>
       </c>
       <c r="B111" s="16" t="s">
         <v>139</v>
@@ -3378,7 +3378,7 @@
       <c r="E111" s="17"/>
       <c r="F111" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G111" s="18" t="b">
         <v>1</v>
@@ -3393,7 +3393,7 @@
     <row r="112" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/traffic-speed</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/traffic-speed</v>
       </c>
       <c r="B112" s="24" t="s">
         <v>141</v>
@@ -3403,7 +3403,7 @@
       <c r="E112" s="22"/>
       <c r="F112" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H112" s="22"/>
       <c r="I112" s="22" t="s">
@@ -3413,7 +3413,7 @@
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/location-and-length-of-traffic-queues</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/location-and-length-of-traffic-queues</v>
       </c>
       <c r="B113" s="8" t="s">
         <v>142</v>
@@ -3421,7 +3421,7 @@
       <c r="C113" s="8"/>
       <c r="F113" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I113" s="1" t="s">
         <v>34</v>
@@ -3430,7 +3430,7 @@
     <row r="114" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="15" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B114,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/current-travel-times</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/current-travel-times</v>
       </c>
       <c r="B114" s="16" t="s">
         <v>143</v>
@@ -3440,14 +3440,14 @@
       <c r="E114" s="17"/>
       <c r="F114" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G114" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H114" s="17" t="str">
         <f>A115</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/current-road-travel-times</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/current-road-travel-times</v>
       </c>
       <c r="I114" s="18" t="s">
         <v>34</v>
@@ -3456,7 +3456,7 @@
     <row r="115" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="20" t="str">
         <f t="shared" ref="A115:A119" si="3">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B115,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/current-road-travel-times</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/current-road-travel-times</v>
       </c>
       <c r="B115" s="24" t="s">
         <v>144</v>
@@ -3466,17 +3466,17 @@
       <c r="E115" s="22"/>
       <c r="F115" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H115" s="22"/>
       <c r="I115" s="23" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="116" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A116" s="15" t="str">
         <f t="shared" si="3"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/predicted-travel-times</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/predicted-travel-times</v>
       </c>
       <c r="B116" s="16" t="s">
         <v>145</v>
@@ -3486,14 +3486,14 @@
       <c r="E116" s="17"/>
       <c r="F116" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G116" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H116" s="17" t="str">
         <f>A117</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/predicted-road-travel-times</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/predicted-road-travel-times</v>
       </c>
       <c r="I116" s="17" t="s">
         <v>34</v>
@@ -3502,7 +3502,7 @@
     <row r="117" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="20" t="str">
         <f t="shared" si="3"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/predicted-road-travel-times</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/predicted-road-travel-times</v>
       </c>
       <c r="B117" s="24" t="s">
         <v>146</v>
@@ -3512,17 +3512,17 @@
       <c r="E117" s="22"/>
       <c r="F117" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H117" s="22"/>
       <c r="I117" s="23" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="118" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A118" s="15" t="str">
         <f t="shared" si="3"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/expected-delays</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/expected-delays</v>
       </c>
       <c r="B118" s="16" t="s">
         <v>147</v>
@@ -3532,14 +3532,14 @@
       <c r="E118" s="17"/>
       <c r="F118" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G118" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H118" s="17" t="str">
         <f>A119</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/expected-road-traffic-delays</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/expected-road-traffic-delays</v>
       </c>
       <c r="I118" s="17" t="s">
         <v>34</v>
@@ -3548,7 +3548,7 @@
     <row r="119" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="20" t="str">
         <f t="shared" si="3"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/expected-road-traffic-delays</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/expected-road-traffic-delays</v>
       </c>
       <c r="B119" s="24" t="s">
         <v>148</v>
@@ -3558,7 +3558,7 @@
       <c r="E119" s="22"/>
       <c r="F119" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H119" s="22"/>
       <c r="I119" s="23" t="s">
@@ -3568,7 +3568,7 @@
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/waiting-time-at-border-crossings-to-non-eu-member-states</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/waiting-time-at-border-crossings-to-non-eu-member-states</v>
       </c>
       <c r="B120" s="8" t="s">
         <v>149</v>
@@ -3576,7 +3576,7 @@
       <c r="C120" s="8"/>
       <c r="F120" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I120" s="1" t="s">
         <v>34</v>
@@ -3585,7 +3585,7 @@
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/traffic-data-at-border-crossings-to-third-countries</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/traffic-data-at-border-crossings-to-third-countries</v>
       </c>
       <c r="B121" s="8" t="s">
         <v>150</v>
@@ -3593,7 +3593,7 @@
       <c r="C121" s="8"/>
       <c r="F121" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I121" s="25" t="s">
         <v>34</v>
@@ -3602,7 +3602,7 @@
     <row r="122" spans="1:9" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/general-information-for-trip-planning</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/general-information-for-trip-planning</v>
       </c>
       <c r="B122" s="9" t="s">
         <v>151</v>
@@ -3610,11 +3610,11 @@
       <c r="C122" s="8"/>
       <c r="E122" s="1" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A123:A129)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/address-identifiers, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/topographic-places, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/points-of-interest, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parameters-needed-to-calculate-environmental-factors, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parameters-needed-to-calculate-costs, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parameters-needed-to-calculate-energy-fuel-consumption, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/estimated-travel-times-for-multimodal-trip-planning</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/address-identifiers, https://w3id.org/mobilitydcat-ap/mobility-theme/topographic-places, https://w3id.org/mobilitydcat-ap/mobility-theme/points-of-interest, https://w3id.org/mobilitydcat-ap/mobility-theme/parameters-needed-to-calculate-environmental-factors, https://w3id.org/mobilitydcat-ap/mobility-theme/parameters-needed-to-calculate-costs, https://w3id.org/mobilitydcat-ap/mobility-theme/parameters-needed-to-calculate-energy-fuel-consumption, https://w3id.org/mobilitydcat-ap/mobility-theme/estimated-travel-times-for-multimodal-trip-planning</v>
       </c>
       <c r="F122" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I122" s="1" t="s">
         <v>46</v>
@@ -3623,7 +3623,7 @@
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/address-identifiers</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/address-identifiers</v>
       </c>
       <c r="B123" s="8" t="s">
         <v>152</v>
@@ -3631,7 +3631,7 @@
       <c r="C123" s="8"/>
       <c r="F123" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I123" s="1" t="s">
         <v>46</v>
@@ -3640,7 +3640,7 @@
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/topographic-places</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/topographic-places</v>
       </c>
       <c r="B124" s="8" t="s">
         <v>153</v>
@@ -3648,7 +3648,7 @@
       <c r="C124" s="8"/>
       <c r="F124" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I124" s="1" t="s">
         <v>46</v>
@@ -3657,7 +3657,7 @@
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/points-of-interest</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/points-of-interest</v>
       </c>
       <c r="B125" s="8" t="s">
         <v>154</v>
@@ -3665,7 +3665,7 @@
       <c r="C125" s="8"/>
       <c r="F125" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I125" s="1" t="s">
         <v>46</v>
@@ -3674,7 +3674,7 @@
     <row r="126" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A126" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parameters-needed-to-calculate-environmental-factors</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parameters-needed-to-calculate-environmental-factors</v>
       </c>
       <c r="B126" s="8" t="s">
         <v>155</v>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="F126" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I126" s="1" t="s">
         <v>46</v>
@@ -3694,7 +3694,7 @@
     <row r="127" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A127" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parameters-needed-to-calculate-costs</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parameters-needed-to-calculate-costs</v>
       </c>
       <c r="B127" s="16" t="s">
         <v>157</v>
@@ -3704,7 +3704,7 @@
       <c r="E127" s="17"/>
       <c r="F127" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G127" s="18" t="b">
         <v>1</v>
@@ -3717,7 +3717,7 @@
     <row r="128" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A128" s="20" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B128,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/parameters-needed-to-calculate-energy-fuel-consumption</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/parameters-needed-to-calculate-energy-fuel-consumption</v>
       </c>
       <c r="B128" s="24" t="s">
         <v>159</v>
@@ -3729,7 +3729,7 @@
       <c r="E128" s="22"/>
       <c r="F128" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H128" s="22"/>
       <c r="I128" s="22" t="s">
@@ -3739,7 +3739,7 @@
     <row r="129" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A129" s="20" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B129,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/estimated-travel-times-for-multimodal-trip-planning</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/estimated-travel-times-for-multimodal-trip-planning</v>
       </c>
       <c r="B129" s="21" t="s">
         <v>161</v>
@@ -3751,7 +3751,7 @@
       <c r="E129" s="22"/>
       <c r="F129" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H129" s="22"/>
       <c r="I129" s="22" t="s">
@@ -3761,7 +3761,7 @@
     <row r="130" spans="1:9" s="18" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="15" t="str">
         <f t="shared" ref="A130" si="4">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B130,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/public-transport-scheduled-transport</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/public-transport-scheduled-transport</v>
       </c>
       <c r="B130" s="16" t="s">
         <v>163</v>
@@ -3771,7 +3771,7 @@
       <c r="E130" s="17"/>
       <c r="F130" s="17" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="G130" s="18" t="b">
         <v>1</v>
@@ -3795,21 +3795,21 @@
       <c r="D131" s="22"/>
       <c r="E131" s="22" t="str">
         <f>_xlfn.TEXTJOIN(" ,",,A133:A174)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-location-and-features ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/stop-facilities-geometry-and-map-layout ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-geometry-and-map-layout ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/stop-facilities-status-of-features ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-features-status ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/stop-facilities-accessibility-and-paths-within-facility ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/accessibility-and-paths-within-facilities ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/operational-calendar ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/connection-links ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/network-topology-and-routes-lines ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/transport-operators ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/timetables-static ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/real-time-estimated-departure-and-arrival-times ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/planned-interchanges-between-scheduled-services ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/hours-of-operation ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/vehicle-details ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/transport-operator-vehicle-fleet-description ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/environmental-standards-for-vehicles ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/disruptions-delays-cancellations ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/basic-common-standard-fares ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/passenger-classes ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/common-fare-products ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/special-fare-products ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/basic-commercial-conditions ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/purchase-information ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/purchase-and-reservation-information ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/defaut-transfer-times-at-interchanges ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/default-transfer-times-at-interchanges ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/existence-of-assistance-services ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/historic-travel-and-traffic-data-and-delays ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/observed-data-on-delays-and-passing-time ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/observed-data-on-cancellations ,https://w3id.org/mobilitydcat-ap/mobility-theme/vehicle-occupancy ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/public-transport-non-scheduled-transport ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/provider-data ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/public-transport-provider-data ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-areas-and-service-times ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-area ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/locations-and-stations ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/fares ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/reservation-and-purchase-options ,https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/accessibility-information-for-vehicles</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/facility-location-and-features ,https://w3id.org/mobilitydcat-ap/mobility-theme/stop-facilities-geometry-and-map-layout ,https://w3id.org/mobilitydcat-ap/mobility-theme/facility-geometry-and-map-layout ,https://w3id.org/mobilitydcat-ap/mobility-theme/stop-facilities-status-of-features ,https://w3id.org/mobilitydcat-ap/mobility-theme/facility-features-status ,https://w3id.org/mobilitydcat-ap/mobility-theme/stop-facilities-accessibility-and-paths-within-facility ,https://w3id.org/mobilitydcat-ap/mobility-theme/accessibility-and-paths-within-facilities ,https://w3id.org/mobilitydcat-ap/mobility-theme/operational-calendar ,https://w3id.org/mobilitydcat-ap/mobility-theme/connection-links ,https://w3id.org/mobilitydcat-ap/mobility-theme/network-topology-and-routes-lines ,https://w3id.org/mobilitydcat-ap/mobility-theme/transport-operators ,https://w3id.org/mobilitydcat-ap/mobility-theme/timetables-static ,https://w3id.org/mobilitydcat-ap/mobility-theme/real-time-estimated-departure-and-arrival-times ,https://w3id.org/mobilitydcat-ap/mobility-theme/planned-interchanges-between-scheduled-services ,https://w3id.org/mobilitydcat-ap/mobility-theme/hours-of-operation ,https://w3id.org/mobilitydcat-ap/mobility-theme/vehicle-details ,https://w3id.org/mobilitydcat-ap/mobility-theme/transport-operator-vehicle-fleet-description ,https://w3id.org/mobilitydcat-ap/mobility-theme/environmental-standards-for-vehicles ,https://w3id.org/mobilitydcat-ap/mobility-theme/disruptions-delays-cancellations ,https://w3id.org/mobilitydcat-ap/mobility-theme/basic-common-standard-fares ,https://w3id.org/mobilitydcat-ap/mobility-theme/passenger-classes ,https://w3id.org/mobilitydcat-ap/mobility-theme/common-fare-products ,https://w3id.org/mobilitydcat-ap/mobility-theme/special-fare-products ,https://w3id.org/mobilitydcat-ap/mobility-theme/basic-commercial-conditions ,https://w3id.org/mobilitydcat-ap/mobility-theme/purchase-information ,https://w3id.org/mobilitydcat-ap/mobility-theme/purchase-and-reservation-information ,https://w3id.org/mobilitydcat-ap/mobility-theme/defaut-transfer-times-at-interchanges ,https://w3id.org/mobilitydcat-ap/mobility-theme/default-transfer-times-at-interchanges ,https://w3id.org/mobilitydcat-ap/mobility-theme/existence-of-assistance-services ,https://w3id.org/mobilitydcat-ap/mobility-theme/historic-travel-and-traffic-data-and-delays ,https://w3id.org/mobilitydcat-ap/mobility-theme/observed-data-on-delays-and-passing-time ,https://w3id.org/mobilitydcat-ap/mobility-theme/observed-data-on-cancellations ,https://w3id.org/mobilitydcat-ap/mobility-theme/vehicle-occupancy ,https://w3id.org/mobilitydcat-ap/mobility-theme/public-transport-non-scheduled-transport ,https://w3id.org/mobilitydcat-ap/mobility-theme/provider-data ,https://w3id.org/mobilitydcat-ap/mobility-theme/public-transport-provider-data ,https://w3id.org/mobilitydcat-ap/mobility-theme/service-areas-and-service-times ,https://w3id.org/mobilitydcat-ap/mobility-theme/service-area ,https://w3id.org/mobilitydcat-ap/mobility-theme/locations-and-stations ,https://w3id.org/mobilitydcat-ap/mobility-theme/fares ,https://w3id.org/mobilitydcat-ap/mobility-theme/reservation-and-purchase-options ,https://w3id.org/mobilitydcat-ap/mobility-theme/accessibility-information-for-vehicles</v>
       </c>
       <c r="F131" s="22" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="H131" s="22"/>
       <c r="I131" s="22" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="132" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A132" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/stop-facilities-location-and-features</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/stop-facilities-location-and-features</v>
       </c>
       <c r="B132" s="16" t="s">
         <v>166</v>
@@ -3819,14 +3819,14 @@
       <c r="E132" s="17"/>
       <c r="F132" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G132" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H132" s="17" t="str">
         <f>A133</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-location-and-features</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/facility-location-and-features</v>
       </c>
       <c r="I132" s="17" t="s">
         <v>46</v>
@@ -3835,7 +3835,7 @@
     <row r="133" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-location-and-features</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/facility-location-and-features</v>
       </c>
       <c r="B133" s="24" t="s">
         <v>167</v>
@@ -3845,17 +3845,17 @@
       <c r="E133" s="22"/>
       <c r="F133" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H133" s="22"/>
       <c r="I133" s="22" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="134" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A134" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/stop-facilities-geometry-and-map-layout</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/stop-facilities-geometry-and-map-layout</v>
       </c>
       <c r="B134" s="16" t="s">
         <v>168</v>
@@ -3865,14 +3865,14 @@
       <c r="E134" s="17"/>
       <c r="F134" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G134" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H134" s="17" t="str">
         <f>A135</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-geometry-and-map-layout</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/facility-geometry-and-map-layout</v>
       </c>
       <c r="I134" s="17" t="s">
         <v>46</v>
@@ -3881,7 +3881,7 @@
     <row r="135" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-geometry-and-map-layout</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/facility-geometry-and-map-layout</v>
       </c>
       <c r="B135" s="24" t="s">
         <v>169</v>
@@ -3891,7 +3891,7 @@
       <c r="E135" s="22"/>
       <c r="F135" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H135" s="22"/>
       <c r="I135" s="22" t="s">
@@ -3901,7 +3901,7 @@
     <row r="136" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/stop-facilities-status-of-features</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/stop-facilities-status-of-features</v>
       </c>
       <c r="B136" s="16" t="s">
         <v>170</v>
@@ -3911,14 +3911,14 @@
       <c r="E136" s="17"/>
       <c r="F136" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G136" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H136" s="17" t="str">
         <f>A137</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-features-status</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/facility-features-status</v>
       </c>
       <c r="I136" s="17" t="s">
         <v>46</v>
@@ -3927,7 +3927,7 @@
     <row r="137" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-features-status</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/facility-features-status</v>
       </c>
       <c r="B137" s="24" t="s">
         <v>171</v>
@@ -3937,7 +3937,7 @@
       <c r="E137" s="22"/>
       <c r="F137" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H137" s="22"/>
       <c r="I137" s="22"/>
@@ -3945,7 +3945,7 @@
     <row r="138" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/stop-facilities-accessibility-and-paths-within-facility</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/stop-facilities-accessibility-and-paths-within-facility</v>
       </c>
       <c r="B138" s="16" t="s">
         <v>172</v>
@@ -3955,14 +3955,14 @@
       <c r="E138" s="17"/>
       <c r="F138" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G138" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H138" s="18" t="str">
         <f>A139</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/accessibility-and-paths-within-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/accessibility-and-paths-within-facilities</v>
       </c>
       <c r="I138" s="17" t="s">
         <v>46</v>
@@ -3971,7 +3971,7 @@
     <row r="139" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/accessibility-and-paths-within-facilities</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/accessibility-and-paths-within-facilities</v>
       </c>
       <c r="B139" s="24" t="s">
         <v>173</v>
@@ -3981,7 +3981,7 @@
       <c r="E139" s="22"/>
       <c r="F139" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H139" s="22"/>
       <c r="I139" s="22"/>
@@ -3989,7 +3989,7 @@
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/operational-calendar</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/operational-calendar</v>
       </c>
       <c r="B140" s="8" t="s">
         <v>174</v>
@@ -3997,7 +3997,7 @@
       <c r="C140" s="8"/>
       <c r="F140" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I140" s="1" t="s">
         <v>46</v>
@@ -4006,7 +4006,7 @@
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/connection-links</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/connection-links</v>
       </c>
       <c r="B141" s="8" t="s">
         <v>175</v>
@@ -4014,7 +4014,7 @@
       <c r="C141" s="8"/>
       <c r="F141" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I141" s="1" t="s">
         <v>46</v>
@@ -4023,7 +4023,7 @@
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/network-topology-and-routes-lines</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/network-topology-and-routes-lines</v>
       </c>
       <c r="B142" s="8" t="s">
         <v>176</v>
@@ -4031,7 +4031,7 @@
       <c r="C142" s="8"/>
       <c r="F142" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I142" s="1" t="s">
         <v>46</v>
@@ -4040,7 +4040,7 @@
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/transport-operators</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/transport-operators</v>
       </c>
       <c r="B143" s="8" t="s">
         <v>177</v>
@@ -4048,7 +4048,7 @@
       <c r="C143" s="8"/>
       <c r="F143" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I143" s="1" t="s">
         <v>46</v>
@@ -4057,7 +4057,7 @@
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/timetables-static</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/timetables-static</v>
       </c>
       <c r="B144" s="8" t="s">
         <v>178</v>
@@ -4065,7 +4065,7 @@
       <c r="C144" s="8"/>
       <c r="F144" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I144" s="1" t="s">
         <v>46</v>
@@ -4074,7 +4074,7 @@
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/real-time-estimated-departure-and-arrival-times</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/real-time-estimated-departure-and-arrival-times</v>
       </c>
       <c r="B145" s="8" t="s">
         <v>179</v>
@@ -4082,7 +4082,7 @@
       <c r="C145" s="8"/>
       <c r="F145" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I145" s="1" t="s">
         <v>46</v>
@@ -4091,7 +4091,7 @@
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/planned-interchanges-between-scheduled-services</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/planned-interchanges-between-scheduled-services</v>
       </c>
       <c r="B146" s="8" t="s">
         <v>180</v>
@@ -4099,16 +4099,16 @@
       <c r="C146" s="8"/>
       <c r="F146" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I146" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A147" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/hours-of-operation</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/hours-of-operation</v>
       </c>
       <c r="B147" s="8" t="s">
         <v>181</v>
@@ -4119,16 +4119,16 @@
       </c>
       <c r="F147" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I147" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="148" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A148" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/vehicle-details</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/vehicle-details</v>
       </c>
       <c r="B148" s="16" t="s">
         <v>183</v>
@@ -4138,14 +4138,14 @@
       <c r="E148" s="17"/>
       <c r="F148" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G148" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H148" s="17" t="str">
         <f>A149</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/transport-operator-vehicle-fleet-description</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/transport-operator-vehicle-fleet-description</v>
       </c>
       <c r="I148" s="17" t="s">
         <v>46</v>
@@ -4154,7 +4154,7 @@
     <row r="149" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A149" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/transport-operator-vehicle-fleet-description</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/transport-operator-vehicle-fleet-description</v>
       </c>
       <c r="B149" s="24" t="s">
         <v>184</v>
@@ -4166,15 +4166,15 @@
       <c r="E149" s="22"/>
       <c r="F149" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H149" s="22"/>
       <c r="I149" s="22"/>
     </row>
-    <row r="150" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A150" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/environmental-standards-for-vehicles</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/environmental-standards-for-vehicles</v>
       </c>
       <c r="B150" s="16" t="s">
         <v>186</v>
@@ -4184,14 +4184,14 @@
       <c r="E150" s="17"/>
       <c r="F150" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G150" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H150" s="17" t="str">
         <f>A149</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/transport-operator-vehicle-fleet-description</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/transport-operator-vehicle-fleet-description</v>
       </c>
       <c r="I150" s="17" t="s">
         <v>46</v>
@@ -4200,7 +4200,7 @@
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="10" t="str">
         <f t="shared" ref="A151:A196" si="5">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B151,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/disruptions-delays-cancellations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/disruptions-delays-cancellations</v>
       </c>
       <c r="B151" s="8" t="s">
         <v>187</v>
@@ -4208,7 +4208,7 @@
       <c r="C151" s="8"/>
       <c r="F151" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I151" s="1" t="s">
         <v>46</v>
@@ -4217,7 +4217,7 @@
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/basic-common-standard-fares</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/basic-common-standard-fares</v>
       </c>
       <c r="B152" s="8" t="s">
         <v>188</v>
@@ -4225,7 +4225,7 @@
       <c r="C152" s="8"/>
       <c r="F152" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I152" s="1" t="s">
         <v>46</v>
@@ -4234,7 +4234,7 @@
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/passenger-classes</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/passenger-classes</v>
       </c>
       <c r="B153" s="8" t="s">
         <v>189</v>
@@ -4242,7 +4242,7 @@
       <c r="C153" s="8"/>
       <c r="F153" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I153" s="1" t="s">
         <v>46</v>
@@ -4251,7 +4251,7 @@
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/common-fare-products</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/common-fare-products</v>
       </c>
       <c r="B154" s="8" t="s">
         <v>190</v>
@@ -4259,7 +4259,7 @@
       <c r="C154" s="8"/>
       <c r="F154" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I154" s="1" t="s">
         <v>46</v>
@@ -4268,7 +4268,7 @@
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/special-fare-products</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/special-fare-products</v>
       </c>
       <c r="B155" s="8" t="s">
         <v>191</v>
@@ -4276,7 +4276,7 @@
       <c r="C155" s="8"/>
       <c r="F155" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I155" s="1" t="s">
         <v>46</v>
@@ -4285,7 +4285,7 @@
     <row r="156" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A156" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/basic-commercial-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/basic-commercial-conditions</v>
       </c>
       <c r="B156" s="8" t="s">
         <v>192</v>
@@ -4296,16 +4296,16 @@
       </c>
       <c r="F156" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I156" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="157" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A157" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/purchase-information</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/purchase-information</v>
       </c>
       <c r="B157" s="16" t="s">
         <v>194</v>
@@ -4315,14 +4315,14 @@
       <c r="E157" s="17"/>
       <c r="F157" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G157" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H157" s="17" t="str">
         <f>A158</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/purchase-and-reservation-information</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/purchase-and-reservation-information</v>
       </c>
       <c r="I157" s="17" t="s">
         <v>46</v>
@@ -4331,7 +4331,7 @@
     <row r="158" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/purchase-and-reservation-information</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/purchase-and-reservation-information</v>
       </c>
       <c r="B158" s="24" t="s">
         <v>195</v>
@@ -4341,17 +4341,17 @@
       <c r="E158" s="22"/>
       <c r="F158" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H158" s="22"/>
       <c r="I158" s="23" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="159" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A159" s="15" t="str">
         <f t="shared" ref="A159" si="6">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B159,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/defaut-transfer-times-at-interchanges</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/defaut-transfer-times-at-interchanges</v>
       </c>
       <c r="B159" s="32" t="s">
         <v>196</v>
@@ -4361,14 +4361,14 @@
       <c r="E159" s="17"/>
       <c r="F159" s="17" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="G159" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H159" s="17" t="str">
         <f>A160</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/default-transfer-times-at-interchanges</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/default-transfer-times-at-interchanges</v>
       </c>
       <c r="I159" s="18" t="s">
         <v>46</v>
@@ -4377,7 +4377,7 @@
     <row r="160" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/default-transfer-times-at-interchanges</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/default-transfer-times-at-interchanges</v>
       </c>
       <c r="B160" s="30" t="s">
         <v>197</v>
@@ -4387,17 +4387,17 @@
       <c r="E160" s="22"/>
       <c r="F160" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H160" s="22"/>
       <c r="I160" s="23" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="161" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A161" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/existence-of-assistance-services</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/existence-of-assistance-services</v>
       </c>
       <c r="B161" s="30" t="s">
         <v>198</v>
@@ -4409,7 +4409,7 @@
       <c r="E161" s="22"/>
       <c r="F161" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H161" s="22"/>
       <c r="I161" s="22" t="s">
@@ -4419,7 +4419,7 @@
     <row r="162" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/historic-travel-and-traffic-data-and-delays</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/historic-travel-and-traffic-data-and-delays</v>
       </c>
       <c r="B162" s="30" t="s">
         <v>200</v>
@@ -4429,7 +4429,7 @@
       <c r="E162" s="22"/>
       <c r="F162" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H162" s="22"/>
       <c r="I162" s="22" t="s">
@@ -4439,7 +4439,7 @@
     <row r="163" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/observed-data-on-delays-and-passing-time</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/observed-data-on-delays-and-passing-time</v>
       </c>
       <c r="B163" s="30" t="s">
         <v>201</v>
@@ -4449,7 +4449,7 @@
       <c r="E163" s="22"/>
       <c r="F163" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H163" s="22"/>
       <c r="I163" s="22" t="s">
@@ -4459,7 +4459,7 @@
     <row r="164" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/observed-data-on-cancellations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/observed-data-on-cancellations</v>
       </c>
       <c r="B164" s="30" t="s">
         <v>202</v>
@@ -4469,14 +4469,14 @@
       <c r="E164" s="22"/>
       <c r="F164" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H164" s="22"/>
       <c r="I164" s="22" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="165" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A165" s="23" t="s">
         <v>203</v>
       </c>
@@ -4490,7 +4490,7 @@
       <c r="E165" s="22"/>
       <c r="F165" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H165" s="22"/>
       <c r="I165" s="22" t="s">
@@ -4500,7 +4500,7 @@
     <row r="166" spans="1:9" s="18" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="15" t="str">
         <f t="shared" ref="A166" si="7">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B166,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/public-transport-non-scheduled-transport</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/public-transport-non-scheduled-transport</v>
       </c>
       <c r="B166" s="16" t="s">
         <v>206</v>
@@ -4510,7 +4510,7 @@
       <c r="E166" s="17"/>
       <c r="F166" s="17" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="G166" s="18" t="b">
         <v>1</v>
@@ -4526,7 +4526,7 @@
     <row r="167" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/provider-data</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/provider-data</v>
       </c>
       <c r="B167" s="16" t="s">
         <v>207</v>
@@ -4536,7 +4536,7 @@
       <c r="E167" s="17"/>
       <c r="F167" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G167" s="18" t="b">
         <v>1</v>
@@ -4551,7 +4551,7 @@
     <row r="168" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/public-transport-provider-data</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/public-transport-provider-data</v>
       </c>
       <c r="B168" s="24" t="s">
         <v>209</v>
@@ -4561,7 +4561,7 @@
       <c r="E168" s="22"/>
       <c r="F168" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H168" s="22"/>
       <c r="I168" s="22" t="s">
@@ -4571,7 +4571,7 @@
     <row r="169" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A169" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-areas-and-service-times</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-areas-and-service-times</v>
       </c>
       <c r="B169" s="16" t="s">
         <v>210</v>
@@ -4581,14 +4581,14 @@
       <c r="E169" s="17"/>
       <c r="F169" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G169" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H169" s="17" t="str">
         <f>_xlfn.CONCAT(A170, ", ",A147)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-area, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/hours-of-operation</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-area, https://w3id.org/mobilitydcat-ap/mobility-theme/hours-of-operation</v>
       </c>
       <c r="I169" s="17" t="s">
         <v>46</v>
@@ -4597,7 +4597,7 @@
     <row r="170" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-area</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-area</v>
       </c>
       <c r="B170" s="24" t="s">
         <v>211</v>
@@ -4607,17 +4607,17 @@
       <c r="E170" s="22"/>
       <c r="F170" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H170" s="22"/>
       <c r="I170" s="31" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="171" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A171" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/locations-and-stations</v>
       </c>
       <c r="B171" s="16" t="s">
         <v>212</v>
@@ -4627,23 +4627,23 @@
       <c r="E171" s="17"/>
       <c r="F171" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G171" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H171" s="17" t="str">
         <f>A133</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/facility-location-and-features</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/facility-location-and-features</v>
       </c>
       <c r="I171" s="18" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="172" spans="1:9" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:9" s="18" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A172" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/fares</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/fares</v>
       </c>
       <c r="B172" s="16" t="s">
         <v>213</v>
@@ -4653,23 +4653,23 @@
       <c r="E172" s="17"/>
       <c r="F172" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G172" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H172" s="17" t="str">
         <f>_xlfn.CONCAT(A153, ", ", _xlfn.TEXTJOIN(", ",,A154:A156))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/passenger-classes, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/common-fare-products, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/special-fare-products, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/basic-commercial-conditions</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/passenger-classes, https://w3id.org/mobilitydcat-ap/mobility-theme/common-fare-products, https://w3id.org/mobilitydcat-ap/mobility-theme/special-fare-products, https://w3id.org/mobilitydcat-ap/mobility-theme/basic-commercial-conditions</v>
       </c>
       <c r="I172" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="173" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A173" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/reservation-and-purchase-options</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/reservation-and-purchase-options</v>
       </c>
       <c r="B173" s="16" t="s">
         <v>214</v>
@@ -4679,14 +4679,14 @@
       <c r="E173" s="17"/>
       <c r="F173" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G173" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H173" s="17" t="str">
         <f>A158</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/purchase-and-reservation-information</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/purchase-and-reservation-information</v>
       </c>
       <c r="I173" s="17" t="s">
         <v>46</v>
@@ -4695,7 +4695,7 @@
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/accessibility-information-for-vehicles</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/accessibility-information-for-vehicles</v>
       </c>
       <c r="B174" s="27" t="s">
         <v>215</v>
@@ -4703,7 +4703,7 @@
       <c r="C174" s="8"/>
       <c r="F174" s="1" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="I174" s="1" t="s">
         <v>46</v>
@@ -4712,7 +4712,7 @@
     <row r="175" spans="1:9" s="18" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/sharing-and-hiring-services</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/sharing-and-hiring-services</v>
       </c>
       <c r="B175" s="16" t="s">
         <v>216</v>
@@ -4722,7 +4722,7 @@
       <c r="E175" s="17"/>
       <c r="F175" s="17" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="H175" s="17"/>
       <c r="I175" s="17" t="s">
@@ -4732,7 +4732,7 @@
     <row r="176" spans="1:9" s="23" customFormat="1" ht="198" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/sharing-hiring-and-renting-services</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/sharing-hiring-and-renting-services</v>
       </c>
       <c r="B176" s="9" t="s">
         <v>217</v>
@@ -4741,19 +4741,19 @@
       <c r="D176" s="22"/>
       <c r="E176" s="22" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A177:A193)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-sharing-locations-and-stations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-sharing-locations-and-stations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-hiring-stations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-hiring-stations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/e-scooter-sharing-locations-and-stations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-sharing-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-sharing-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-hiring-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-hiring-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/e-scooter-sharing-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-locations-and-stations, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-real-time-availability, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-payment-methods, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-zones, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/payment-methods, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/environmental-standards-for-vehicles</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/bike-sharing-locations-and-stations, https://w3id.org/mobilitydcat-ap/mobility-theme/car-sharing-locations-and-stations, https://w3id.org/mobilitydcat-ap/mobility-theme/bike-hiring-stations, https://w3id.org/mobilitydcat-ap/mobility-theme/car-hiring-stations, https://w3id.org/mobilitydcat-ap/mobility-theme/e-scooter-sharing-locations-and-stations, https://w3id.org/mobilitydcat-ap/mobility-theme/car-sharing-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/bike-sharing-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/car-hiring-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/bike-hiring-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/e-scooter-sharing-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/service-locations-and-stations, https://w3id.org/mobilitydcat-ap/mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/mobility-theme/service-real-time-availability, https://w3id.org/mobilitydcat-ap/mobility-theme/service-payment-methods, https://w3id.org/mobilitydcat-ap/mobility-theme/service-zones, https://w3id.org/mobilitydcat-ap/mobility-theme/payment-methods, https://w3id.org/mobilitydcat-ap/mobility-theme/environmental-standards-for-vehicles</v>
       </c>
       <c r="F176" s="22" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="H176" s="22"/>
       <c r="I176" s="22"/>
     </row>
-    <row r="177" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A177" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-sharing-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/bike-sharing-locations-and-stations</v>
       </c>
       <c r="B177" s="16" t="s">
         <v>218</v>
@@ -4763,23 +4763,23 @@
       <c r="E177" s="17"/>
       <c r="F177" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G177" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H177" s="17" t="str">
         <f>A187</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-locations-and-stations</v>
       </c>
       <c r="I177" s="18" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="178" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A178" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-sharing-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/car-sharing-locations-and-stations</v>
       </c>
       <c r="B178" s="16" t="s">
         <v>219</v>
@@ -4789,23 +4789,23 @@
       <c r="E178" s="17"/>
       <c r="F178" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G178" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H178" s="17" t="str">
         <f>A187</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-locations-and-stations</v>
       </c>
       <c r="I178" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="179" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A179" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-hiring-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/bike-hiring-stations</v>
       </c>
       <c r="B179" s="16" t="s">
         <v>220</v>
@@ -4815,23 +4815,23 @@
       <c r="E179" s="17"/>
       <c r="F179" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G179" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H179" s="17" t="str">
         <f>A187</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-locations-and-stations</v>
       </c>
       <c r="I179" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="180" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A180" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-hiring-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/car-hiring-stations</v>
       </c>
       <c r="B180" s="16" t="s">
         <v>221</v>
@@ -4841,23 +4841,23 @@
       <c r="E180" s="17"/>
       <c r="F180" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G180" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H180" s="17" t="str">
         <f>A187</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-locations-and-stations</v>
       </c>
       <c r="I180" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="181" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A181" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/e-scooter-sharing-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/e-scooter-sharing-locations-and-stations</v>
       </c>
       <c r="B181" s="16" t="s">
         <v>222</v>
@@ -4867,14 +4867,14 @@
       <c r="E181" s="17"/>
       <c r="F181" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G181" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H181" s="17" t="str">
         <f>A187</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-locations-and-stations</v>
       </c>
       <c r="I181" s="17" t="s">
         <v>46</v>
@@ -4883,7 +4883,7 @@
     <row r="182" spans="1:9" s="18" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-sharing-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/car-sharing-availability</v>
       </c>
       <c r="B182" s="16" t="s">
         <v>223</v>
@@ -4893,23 +4893,23 @@
       <c r="E182" s="17"/>
       <c r="F182" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G182" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H182" s="17" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A188,A189)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/mobility-theme/service-real-time-availability</v>
       </c>
       <c r="I182" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="183" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:9" s="18" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A183" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-sharing-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/bike-sharing-availability</v>
       </c>
       <c r="B183" s="16" t="s">
         <v>224</v>
@@ -4919,23 +4919,23 @@
       <c r="E183" s="17"/>
       <c r="F183" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G183" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H183" s="17" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A188,A189)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/mobility-theme/service-real-time-availability</v>
       </c>
       <c r="I183" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="184" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:9" s="18" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A184" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/car-hiring-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/car-hiring-availability</v>
       </c>
       <c r="B184" s="16" t="s">
         <v>225</v>
@@ -4945,23 +4945,23 @@
       <c r="E184" s="17"/>
       <c r="F184" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G184" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H184" s="17" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A188,A189)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/mobility-theme/service-real-time-availability</v>
       </c>
       <c r="I184" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="185" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:9" s="18" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A185" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/bike-hiring-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/bike-hiring-availability</v>
       </c>
       <c r="B185" s="16" t="s">
         <v>226</v>
@@ -4971,23 +4971,23 @@
       <c r="E185" s="17"/>
       <c r="F185" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G185" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H185" s="17" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A188,A189)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/mobility-theme/service-real-time-availability</v>
       </c>
       <c r="I185" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="186" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:9" s="18" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A186" s="15" t="str">
         <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(SUBSTITUTE(B186,"/","-"))," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/e-scooter-sharing-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/e-scooter-sharing-availability</v>
       </c>
       <c r="B186" s="16" t="s">
         <v>227</v>
@@ -4997,14 +4997,14 @@
       <c r="E186" s="17"/>
       <c r="F186" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G186" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H186" s="17" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A188,A189)</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-vehicle-fleet-description, https://w3id.org/mobilitydcat-ap/mobility-theme/service-real-time-availability</v>
       </c>
       <c r="I186" s="17" t="s">
         <v>46</v>
@@ -5013,7 +5013,7 @@
     <row r="187" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-locations-and-stations</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-locations-and-stations</v>
       </c>
       <c r="B187" s="33" t="s">
         <v>228</v>
@@ -5023,7 +5023,7 @@
       <c r="E187" s="22"/>
       <c r="F187" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H187" s="22"/>
       <c r="I187" s="22" t="s">
@@ -5033,7 +5033,7 @@
     <row r="188" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A188" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-vehicle-fleet-description</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-vehicle-fleet-description</v>
       </c>
       <c r="B188" s="24" t="s">
         <v>229</v>
@@ -5045,7 +5045,7 @@
       <c r="E188" s="22"/>
       <c r="F188" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H188" s="22"/>
       <c r="I188" s="22" t="s">
@@ -5055,7 +5055,7 @@
     <row r="189" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-real-time-availability</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-real-time-availability</v>
       </c>
       <c r="B189" s="24" t="s">
         <v>231</v>
@@ -5065,7 +5065,7 @@
       <c r="E189" s="22"/>
       <c r="F189" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H189" s="22"/>
       <c r="I189" s="22" t="s">
@@ -5075,7 +5075,7 @@
     <row r="190" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-payment-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-payment-methods</v>
       </c>
       <c r="B190" s="24" t="s">
         <v>232</v>
@@ -5085,7 +5085,7 @@
       <c r="E190" s="22"/>
       <c r="F190" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H190" s="22"/>
       <c r="I190" s="22" t="s">
@@ -5095,7 +5095,7 @@
     <row r="191" spans="1:9" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A191" s="20" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-zones</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-zones</v>
       </c>
       <c r="B191" s="21" t="s">
         <v>233</v>
@@ -5107,7 +5107,7 @@
       <c r="E191" s="22"/>
       <c r="F191" s="22" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="H191" s="22"/>
       <c r="I191" s="22" t="s">
@@ -5117,7 +5117,7 @@
     <row r="192" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/payment-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/payment-methods</v>
       </c>
       <c r="B192" s="16" t="s">
         <v>235</v>
@@ -5127,23 +5127,23 @@
       <c r="E192" s="17"/>
       <c r="F192" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G192" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H192" s="17" t="str">
         <f>A190</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-payment-methods</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-payment-methods</v>
       </c>
       <c r="I192" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="193" spans="1:9" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:9" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A193" s="15" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/environmental-standards-for-vehicles</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/environmental-standards-for-vehicles</v>
       </c>
       <c r="B193" s="16" t="s">
         <v>186</v>
@@ -5153,21 +5153,21 @@
       <c r="E193" s="17"/>
       <c r="F193" s="17" t="str">
         <f>A21</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-sub-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-sub-category</v>
       </c>
       <c r="G193" s="18" t="b">
         <v>1</v>
       </c>
       <c r="H193" s="17" t="str">
         <f>A188</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/service-vehicle-fleet-description</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/service-vehicle-fleet-description</v>
       </c>
       <c r="I193" s="17"/>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/air-and-space-travel</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/air-and-space-travel</v>
       </c>
       <c r="B194" s="9" t="s">
         <v>236</v>
@@ -5175,7 +5175,7 @@
       <c r="C194" s="8"/>
       <c r="F194" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I194" s="1" t="s">
         <v>46</v>
@@ -5184,7 +5184,7 @@
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/waterways-and-water-bodies</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/waterways-and-water-bodies</v>
       </c>
       <c r="B195" s="9" t="s">
         <v>237</v>
@@ -5192,7 +5192,7 @@
       <c r="C195" s="8"/>
       <c r="F195" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
       <c r="I195" s="1" t="s">
         <v>46</v>
@@ -5201,7 +5201,7 @@
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A196" s="10" t="str">
         <f t="shared" si="5"/>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/other</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/other</v>
       </c>
       <c r="B196" s="9" t="s">
         <v>238</v>
@@ -5209,7 +5209,7 @@
       <c r="C196" s="8"/>
       <c r="F196" s="1" t="str">
         <f>A20</f>
-        <v>https://w3id.org/mobilitydcat-ap/[candidate-release]-mobility-theme/data-content-category</v>
+        <v>https://w3id.org/mobilitydcat-ap/mobility-theme/data-content-category</v>
       </c>
     </row>
   </sheetData>
@@ -5374,26 +5374,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006748505E66128D48AAED90CD5CD3616F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b912ec8155dd4e933917767331a7e7b9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa" xmlns:ns3="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f994fb40b965d01e7e08c4f92ceb61cd" ns2:_="" ns3:_="">
     <xsd:import namespace="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
@@ -5594,26 +5574,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F704F36C-6F34-42D8-A9E1-097741891E9D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="13e36eaf-61a1-47aa-b343-0f7d626aa9a0"/>
-    <ds:schemaRef ds:uri="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354E852E-38F4-443F-ABCC-E4BE2043727A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4E03DED-ABA6-41DC-A9F2-F03B3D97B70D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5630,4 +5611,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354E852E-38F4-443F-ABCC-E4BE2043727A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F704F36C-6F34-42D8-A9E1-097741891E9D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="13e36eaf-61a1-47aa-b343-0f7d626aa9a0"/>
+    <ds:schemaRef ds:uri="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>